<commit_message>
Integrate real financial datasets
</commit_message>
<xml_diff>
--- a/output/screener_output.xlsx
+++ b/output/screener_output.xlsx
@@ -1349,7 +1349,11 @@
           <t>ADANIPOWER</t>
         </is>
       </c>
-      <c r="AI6" t="inlineStr"/>
+      <c r="AI6" t="inlineStr">
+        <is>
+          <t>Adani Power Ltd</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1432,7 +1436,8 @@
       </c>
       <c r="AI7" t="inlineStr">
         <is>
-          <t>Apollo Hospitals</t>
+          <t>Apollo Hospitals
+Chain of Indian private hospitals</t>
         </is>
       </c>
     </row>
@@ -1517,7 +1522,8 @@
       </c>
       <c r="AI8" t="inlineStr">
         <is>
-          <t>Asian Paints</t>
+          <t>Asian Paints
+Indian Multi-National Paint and Coating Manufacturing Company</t>
         </is>
       </c>
     </row>
@@ -2909,7 +2915,11 @@
           <t>HDFCBANK</t>
         </is>
       </c>
-      <c r="AI24" t="inlineStr"/>
+      <c r="AI24" t="inlineStr">
+        <is>
+          <t>HDFC Bank Ltd</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -3427,7 +3437,11 @@
           <t>INDIGO</t>
         </is>
       </c>
-      <c r="AI30" t="inlineStr"/>
+      <c r="AI30" t="inlineStr">
+        <is>
+          <t>Interglobe Aviation Ltd</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">

</xml_diff>